<commit_message>
Insurgentes SD: roof walls (+30.55) added to the Armado sheet
19 roof wall types ('ROOF - TECHOS' details) moved from the reference
sheet to Armado at elevation +30.55. End elements (free / intersection /
L corner) assigned from the label and dimension positions in the DWG;
each row notes what the detail shows so it can be checked in Revisar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mu9wxeehZ5MxBaqNG8frbT
</commit_message>
<xml_diff>
--- a/revit/ArmadoMuros_Insurgentes/Armado muros (todos los niveles).xlsx
+++ b/revit/ArmadoMuros_Insurgentes/Armado muros (todos los niveles).xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:O80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4268,6 +4268,982 @@
       <c r="O61" s="2" t="inlineStr">
         <is>
           <t>Plano: MURO M-27 N7-ROOF; Geometría (muros/longitudes/alto) tomada de N2, solo referencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-1</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="n"/>
+      <c r="F62" s="3" t="n"/>
+      <c r="G62" s="2" t="n"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>6#4 30 1E+1G@15</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>22#6 200 5E+1G@15</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>40#6 200/200 10E@15</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="n"/>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. En el detalle: 22#6 5E+1G Lb 200, 40#6 10E Lb 200 (dos cotas de 200), ramas de 6#4 1E+1G Lb 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-8</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n"/>
+      <c r="F63" s="3" t="n"/>
+      <c r="G63" s="2" t="n"/>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>8#4 40 2E@15</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="n"/>
+      <c r="L63" s="2" t="n"/>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="n"/>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Ambos extremos 8#4 2E; cotas 40 y 30 en cada extremo: se tomó Lb 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-10</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n"/>
+      <c r="F64" s="3" t="n"/>
+      <c r="G64" s="2" t="n"/>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>6#4 30 1E+1G@15</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>8#4 30 2E@15</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="n"/>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="n"/>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Dos dibujos: extremos 6#4 1E+1G y uno 8#4 2E, todos Lb 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-11 Nivel -2.65</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n"/>
+      <c r="F65" s="3" t="n"/>
+      <c r="G65" s="2" t="n"/>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>12#4 100 3E@15</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>14#4 100 3E+1G@15</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="n"/>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="n"/>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Extremos distintos 12#4 3E / 14#4 3E+1G (Lb 100); el 22#6 5E Lb 185 del detalle es de otro muro</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-12 Nivel -2.65</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="n"/>
+      <c r="F66" s="3" t="n"/>
+      <c r="G66" s="2" t="n"/>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>8#4 60 2E@15</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="n"/>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>10#4 60/40 2E+1G@15</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="n"/>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. 10#4 2E+1G con cotas 60 y 40 (esquina); otro extremo 8#4 2E Lb 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-13 Nivel -2.65</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67" s="3" t="n"/>
+      <c r="G67" s="2" t="n"/>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>12#4 100 3E@15</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>16#4 100 3E+2G@15</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="n"/>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="n"/>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Extremos 16#4 3E+2G / 12#4 3E (Lb 100); ramas: 8#4 2E Lb 60 y 6#4 1E Lb 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-14</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="n"/>
+      <c r="F68" s="3" t="n"/>
+      <c r="G68" s="2" t="n"/>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>14#4 120 3E+1G@15</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="n"/>
+      <c r="L68" s="2" t="n"/>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="n"/>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Ambos extremos 14#4 3E+1G Lb 120; el 22#6 5E+1G Lb 200 del detalle es de la esquina con otro muro</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-15</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n"/>
+      <c r="F69" s="3" t="n"/>
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>6#4 30 1E+1G@15</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>14#6+2#4 120 4E@15</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>32#6 200/120 8E@15</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="n"/>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. 14#6+2#4 4E Lb 120; 32#6 8E con cotas 120 y 200 (esquina); rama 6#4 1E+1G Lb 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-28</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="n"/>
+      <c r="F70" s="3" t="n"/>
+      <c r="G70" s="2" t="n"/>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>16#4 100 3E+2G@15</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="n"/>
+      <c r="L70" s="2" t="n"/>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="n"/>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Ambos extremos 16#4 3E+2G Lb 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-29</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="n"/>
+      <c r="F71" s="3" t="n"/>
+      <c r="G71" s="2" t="n"/>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>14#4 100 3E+1G@15</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="n"/>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>12#4 100/60 2E+1G@15</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="n"/>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. 12#4 2E+1G Lb 100 junto a cotas 60 (esquina con M-1); 14#4 3E+1G Lb 100; rama 6#4 1E+1G Lb 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-30</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n"/>
+      <c r="F72" s="3" t="n"/>
+      <c r="G72" s="2" t="n"/>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>8#4 60 1E+1G@15</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>8#4 60 2E@15</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="n"/>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="n"/>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Ambos extremos 8#4 1E+1G Lb 60; rama 8#4 2E Lb 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-31</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="n"/>
+      <c r="F73" s="3" t="n"/>
+      <c r="G73" s="2" t="n"/>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>6#4 30 1E+1G@15</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>8#4 30 2E@15</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="n"/>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="n"/>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Detalle "M-31 Y M-33": 8#4 2E y 6#4 1E+1G, Lb 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-31A</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="n"/>
+      <c r="F74" s="3" t="n"/>
+      <c r="G74" s="2" t="n"/>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>6#4 30 1E@15</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>8#4 30 2E@15</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="n"/>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="n"/>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Detalle "M-31A Y M-33": 8#4 2E y 6#4 1E, Lb 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-32</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="n"/>
+      <c r="F75" s="3" t="n"/>
+      <c r="G75" s="2" t="n"/>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>6#4 40 1E@15</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>6#4 40 1E+1G@15</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="n"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="n"/>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Extremos 6#4 1E+1G / 6#4 1E, Lb 40; rama 8#4 2E</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-33</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="n"/>
+      <c r="F76" s="3" t="n"/>
+      <c r="G76" s="2" t="n"/>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>6#4 30 1E+1G@15</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>8#4 30 2E@15</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="n"/>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="n"/>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Aparece en "M-31 Y M-33" (6#4 1E+1G) y "M-31A Y M-33" (6#4 1E): se tomó 1E+1G</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-33A</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="n"/>
+      <c r="F77" s="3" t="n"/>
+      <c r="G77" s="2" t="n"/>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>6#6 30 1E+1G@15</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="n"/>
+      <c r="L77" s="2" t="n"/>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="n"/>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Detalle "M-36 Y M-33A": 6#6 1E+1G Lb 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-34</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="n"/>
+      <c r="F78" s="3" t="n"/>
+      <c r="G78" s="2" t="n"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>6#4 40 1E+1G@15</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="n"/>
+      <c r="L78" s="2" t="n"/>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="n"/>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Ambos extremos 6#4 1E+1G Lb 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-35</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="n"/>
+      <c r="F79" s="3" t="n"/>
+      <c r="G79" s="2" t="n"/>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>6#4 30 1E@15</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>6#4 30 1E+1G@15</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="n"/>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="n"/>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Extremos 6#4 1E+1G / 6#4 1E, Lb 30; rama 6#6 1E+1G</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>+30.55</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Muro M-36</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="n"/>
+      <c r="F80" s="3" t="n"/>
+      <c r="G80" s="2" t="n"/>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>#3@30</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>6#4 30 1E@15</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>8#6 30 2E@15</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="n"/>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>E#3 @15</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="n"/>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>Azotea (ROOF-TECHOS, +30.55), leída del DWG: extremos asignados por la posición de las etiquetas, REVISAR en el reporte. Detalle "M-36 Y M-33A": 6#4 1E y 8#6 2E, Lb 30</t>
         </is>
       </c>
     </row>
@@ -4845,7 +5821,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Muros de azotea ("ROOF - TECHOS", arrancan en Roof N10 +30.55). Datos leídos del DWG Muros_I121, SIN asignar a extremos: pasar a la hoja Armado cuando la azotea esté modelada. El botón no lee esta hoja.</t>
+          <t>Datos de azotea leídos del DWG (referencia). YA PASADOS a la hoja Armado (filas +30.55). El botón no lee esta hoja.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Walls: no base leg where the bar continues from the wall below; steel level = level above
- aw_revit: below_walls() finds parallel walls whose crown reaches this wall's base
  (or the underside of the slab between them); aw_geom starts those verticals at
  the base without a leg so they lap with the starter bars from below.
- ArmadoMurosExcel: new setting 'Nivel del acero' (default Superior). The level
  parameter on the bars and the assembly name use the level above the storey
  (top constraint, or the first level at the wall crown), as the plans show the
  plan seen from below. 'Base' keeps the previous behaviour.
- Insurgentes Excel: Configuracion row 'Nivel del acero = Superior'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mu9wxeehZ5MxBaqNG8frbT
</commit_message>
<xml_diff>
--- a/revit/ArmadoMuros_Insurgentes/Armado muros (todos los niveles).xlsx
+++ b/revit/ArmadoMuros_Insurgentes/Armado muros (todos los niveles).xlsx
@@ -5259,7 +5259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -5609,6 +5609,23 @@
       <c r="C21" s="2" t="inlineStr">
         <is>
           <t>{muro} = M-1; {elev} = +16.10; {nivel} = nombre del nivel</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Nivel del acero</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Superior = el acero pertenece al nivel de arriba del entrepiso (muros de +4.70 a +7.55 -&gt; +7.55); Base = nivel de arranque</t>
         </is>
       </c>
     </row>

</xml_diff>